<commit_message>
Still working on analyses
</commit_message>
<xml_diff>
--- a/notebooks/paper_2025/table_3.xlsx
+++ b/notebooks/paper_2025/table_3.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,27 +367,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>design</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NS_11</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>NS_12</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>SSR_11</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SSR_12</t>
+          <t>n_individ</t>
         </is>
       </c>
     </row>
@@ -402,20 +387,13 @@
           <t>hookworm</t>
         </is>
       </c>
-      <c r="C2">
-        <v>0.8</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D2">
-        <v>235</v>
-      </c>
-      <c r="E2">
-        <v>195</v>
-      </c>
-      <c r="F2">
-        <v>350</v>
-      </c>
-      <c r="G2">
-        <v>310</v>
+        <v>615</v>
       </c>
     </row>
     <row r="3">
@@ -429,20 +407,13 @@
           <t>hookworm</t>
         </is>
       </c>
-      <c r="C3">
-        <v>0.9</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D3">
-        <v>355</v>
-      </c>
-      <c r="E3">
-        <v>310</v>
-      </c>
-      <c r="F3">
-        <v>510</v>
-      </c>
-      <c r="G3">
-        <v>460</v>
+        <v>775</v>
       </c>
     </row>
     <row r="4">
@@ -456,20 +427,13 @@
           <t>ascaris</t>
         </is>
       </c>
-      <c r="C4">
-        <v>0.8</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D4">
-        <v>55</v>
-      </c>
-      <c r="E4">
-        <v>35</v>
-      </c>
-      <c r="F4">
-        <v>70</v>
-      </c>
-      <c r="G4">
-        <v>50</v>
+        <v>665</v>
       </c>
     </row>
     <row r="5">
@@ -483,20 +447,13 @@
           <t>ascaris</t>
         </is>
       </c>
-      <c r="C5">
-        <v>0.9</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D5">
-        <v>70</v>
-      </c>
-      <c r="E5">
-        <v>50</v>
-      </c>
-      <c r="F5">
-        <v>90</v>
-      </c>
-      <c r="G5">
-        <v>70</v>
+        <v>670</v>
       </c>
     </row>
     <row r="6">
@@ -510,20 +467,13 @@
           <t>trichuris</t>
         </is>
       </c>
-      <c r="C6">
-        <v>0.8</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D6">
-        <v>5585</v>
-      </c>
-      <c r="E6">
-        <v>5440</v>
-      </c>
-      <c r="F6">
-        <v>6950</v>
-      </c>
-      <c r="G6">
-        <v>6665</v>
+        <v>680</v>
       </c>
     </row>
     <row r="7">
@@ -537,20 +487,13 @@
           <t>trichuris</t>
         </is>
       </c>
-      <c r="C7">
-        <v>0.9</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D7">
-        <v>7300</v>
-      </c>
-      <c r="E7">
-        <v>7115</v>
-      </c>
-      <c r="F7">
-        <v>9200</v>
-      </c>
-      <c r="G7">
-        <v>8790</v>
+        <v>825</v>
       </c>
     </row>
     <row r="8">
@@ -564,20 +507,13 @@
           <t>hookworm</t>
         </is>
       </c>
-      <c r="C8">
-        <v>0.8</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D8">
-        <v>2915</v>
-      </c>
-      <c r="E8">
-        <v>2840</v>
-      </c>
-      <c r="F8">
-        <v>3625</v>
-      </c>
-      <c r="G8">
-        <v>3575</v>
+        <v>665</v>
       </c>
     </row>
     <row r="9">
@@ -591,20 +527,13 @@
           <t>hookworm</t>
         </is>
       </c>
-      <c r="C9">
-        <v>0.9</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D9">
-        <v>3980</v>
-      </c>
-      <c r="E9">
-        <v>3820</v>
-      </c>
-      <c r="F9">
-        <v>5000</v>
-      </c>
-      <c r="G9">
-        <v>4870</v>
+        <v>825</v>
       </c>
     </row>
     <row r="10">
@@ -618,20 +547,13 @@
           <t>ascaris</t>
         </is>
       </c>
-      <c r="C10">
-        <v>0.8</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D10">
-        <v>205</v>
-      </c>
-      <c r="E10">
-        <v>195</v>
-      </c>
-      <c r="F10">
-        <v>255</v>
-      </c>
-      <c r="G10">
-        <v>250</v>
+        <v>750</v>
       </c>
     </row>
     <row r="11">
@@ -645,20 +567,13 @@
           <t>ascaris</t>
         </is>
       </c>
-      <c r="C11">
-        <v>0.9</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D11">
-        <v>335</v>
-      </c>
-      <c r="E11">
-        <v>335</v>
-      </c>
-      <c r="F11">
-        <v>415</v>
-      </c>
-      <c r="G11">
-        <v>415</v>
+        <v>855</v>
       </c>
     </row>
     <row r="12">
@@ -672,20 +587,13 @@
           <t>trichuris</t>
         </is>
       </c>
-      <c r="C12">
-        <v>0.8</v>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NS_11</t>
+        </is>
       </c>
       <c r="D12">
-        <v>6055</v>
-      </c>
-      <c r="E12">
-        <v>5945</v>
-      </c>
-      <c r="F12">
-        <v>7485</v>
-      </c>
-      <c r="G12">
-        <v>7360</v>
+        <v>655</v>
       </c>
     </row>
     <row r="13">
@@ -699,20 +607,13 @@
           <t>trichuris</t>
         </is>
       </c>
-      <c r="C13">
-        <v>0.9</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SSR_12</t>
+        </is>
       </c>
       <c r="D13">
-        <v>7910</v>
-      </c>
-      <c r="E13">
-        <v>7770</v>
-      </c>
-      <c r="F13">
-        <v>9905</v>
-      </c>
-      <c r="G13">
-        <v>9735</v>
+        <v>810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>